<commit_message>
GL-4 DD_GINI_P1 small change to keep consistent with P2
</commit_message>
<xml_diff>
--- a/rmonize/data_dictionary/DD_GINI_P1.xlsx
+++ b/rmonize/data_dictionary/DD_GINI_P1.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20417"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="H:\Projekte\NFDI4Health\TA5\Pilotprojekte\Harmonisierung\HarmonizR\use-cases-harmonisation\rmonize\data_dictionary\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="K:\use-cases-harmonisation\rmonize\data_dictionary\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F3336BE2-AF4B-45D8-903B-1182C1C9CDED}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A0E3838A-CD85-47E3-AEB3-41F2C7F662EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12228" xr2:uid="{1200B70D-B446-4CDA-99A8-3FD394D791D2}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="22290" windowHeight="12000" activeTab="1" xr2:uid="{1200B70D-B446-4CDA-99A8-3FD394D791D2}"/>
   </bookViews>
   <sheets>
     <sheet name="Variables" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="331" uniqueCount="213">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="331" uniqueCount="212">
   <si>
     <t>index</t>
   </si>
@@ -603,9 +603,6 @@
   </si>
   <si>
     <t>Sonstiger Abschluss</t>
-  </si>
-  <si>
-    <t>kein Abschluss</t>
   </si>
   <si>
     <t>Hochschule/Fachhochschuli/Universität</t>
@@ -771,7 +768,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Standard" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -787,9 +784,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -827,7 +824,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -933,7 +930,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1075,7 +1072,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -1084,14 +1081,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{08A73012-5CAD-43B9-A281-79101DF4E1E0}">
   <dimension ref="A1:D96"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.44140625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="19.109375" customWidth="1"/>
-    <col min="3" max="3" width="53.44140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="11.5546875"/>
+    <col min="2" max="2" width="19.140625" customWidth="1"/>
+    <col min="3" max="3" width="53.42578125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.5703125"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1105,12 +1102,12 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="C2" s="6" t="s">
         <v>4</v>
@@ -1119,7 +1116,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2</v>
       </c>
@@ -1133,7 +1130,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>3</v>
       </c>
@@ -1147,7 +1144,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>4</v>
       </c>
@@ -1161,7 +1158,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>5</v>
       </c>
@@ -1175,91 +1172,91 @@
         <v>5</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>6</v>
       </c>
       <c r="B7" t="s">
+        <v>200</v>
+      </c>
+      <c r="C7" t="s">
         <v>201</v>
       </c>
-      <c r="C7" t="s">
-        <v>202</v>
-      </c>
       <c r="D7" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>7</v>
       </c>
       <c r="B8" t="s">
+        <v>202</v>
+      </c>
+      <c r="C8" t="s">
         <v>203</v>
       </c>
-      <c r="C8" t="s">
-        <v>204</v>
-      </c>
       <c r="D8" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>8</v>
       </c>
       <c r="B9" t="s">
+        <v>204</v>
+      </c>
+      <c r="C9" t="s">
         <v>205</v>
       </c>
-      <c r="C9" t="s">
-        <v>206</v>
-      </c>
       <c r="D9" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>9</v>
       </c>
       <c r="B10" t="s">
+        <v>206</v>
+      </c>
+      <c r="C10" t="s">
         <v>207</v>
       </c>
-      <c r="C10" t="s">
-        <v>208</v>
-      </c>
       <c r="D10" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>10</v>
       </c>
       <c r="B11" t="s">
+        <v>208</v>
+      </c>
+      <c r="C11" t="s">
         <v>209</v>
       </c>
-      <c r="C11" t="s">
-        <v>210</v>
-      </c>
       <c r="D11" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>11</v>
       </c>
       <c r="B12" t="s">
+        <v>210</v>
+      </c>
+      <c r="C12" t="s">
         <v>211</v>
       </c>
-      <c r="C12" t="s">
-        <v>212</v>
-      </c>
       <c r="D12" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>12</v>
       </c>
@@ -1273,7 +1270,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>13</v>
       </c>
@@ -1287,7 +1284,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>14</v>
       </c>
@@ -1301,7 +1298,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>15</v>
       </c>
@@ -1315,7 +1312,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>16</v>
       </c>
@@ -1329,7 +1326,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>17</v>
       </c>
@@ -1343,7 +1340,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>18</v>
       </c>
@@ -1357,7 +1354,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>19</v>
       </c>
@@ -1371,7 +1368,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>20</v>
       </c>
@@ -1385,7 +1382,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>21</v>
       </c>
@@ -1399,7 +1396,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>22</v>
       </c>
@@ -1413,7 +1410,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>23</v>
       </c>
@@ -1427,7 +1424,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A25">
         <v>24</v>
       </c>
@@ -1441,7 +1438,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A26">
         <v>25</v>
       </c>
@@ -1455,7 +1452,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A27">
         <v>26</v>
       </c>
@@ -1469,7 +1466,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A28">
         <v>27</v>
       </c>
@@ -1483,7 +1480,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A29">
         <v>28</v>
       </c>
@@ -1497,7 +1494,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A30">
         <v>29</v>
       </c>
@@ -1511,7 +1508,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A31">
         <v>30</v>
       </c>
@@ -1525,7 +1522,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A32">
         <v>31</v>
       </c>
@@ -1539,7 +1536,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A33">
         <v>32</v>
       </c>
@@ -1553,7 +1550,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A34">
         <v>33</v>
       </c>
@@ -1567,7 +1564,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A35">
         <v>34</v>
       </c>
@@ -1581,7 +1578,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A36">
         <v>35</v>
       </c>
@@ -1595,7 +1592,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A37">
         <v>36</v>
       </c>
@@ -1609,7 +1606,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A38">
         <v>37</v>
       </c>
@@ -1623,7 +1620,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A39">
         <v>38</v>
       </c>
@@ -1637,7 +1634,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A40">
         <v>39</v>
       </c>
@@ -1651,7 +1648,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A41">
         <v>40</v>
       </c>
@@ -1665,7 +1662,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A42">
         <v>41</v>
       </c>
@@ -1679,7 +1676,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A43">
         <v>42</v>
       </c>
@@ -1693,7 +1690,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A44">
         <v>43</v>
       </c>
@@ -1707,7 +1704,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A45">
         <v>44</v>
       </c>
@@ -1721,7 +1718,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A46">
         <v>45</v>
       </c>
@@ -1735,7 +1732,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A47">
         <v>46</v>
       </c>
@@ -1749,7 +1746,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="48" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A48">
         <v>47</v>
       </c>
@@ -1763,7 +1760,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A49">
         <v>48</v>
       </c>
@@ -1777,7 +1774,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="50" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A50">
         <v>49</v>
       </c>
@@ -1791,7 +1788,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="51" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A51">
         <v>50</v>
       </c>
@@ -1805,7 +1802,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="52" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A52">
         <v>51</v>
       </c>
@@ -1819,7 +1816,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="53" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A53">
         <v>52</v>
       </c>
@@ -1833,7 +1830,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="54" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A54">
         <v>53</v>
       </c>
@@ -1847,7 +1844,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="55" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A55">
         <v>54</v>
       </c>
@@ -1861,7 +1858,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="56" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A56">
         <v>55</v>
       </c>
@@ -1875,7 +1872,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="57" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A57">
         <v>56</v>
       </c>
@@ -1889,7 +1886,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="58" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A58">
         <v>57</v>
       </c>
@@ -1903,7 +1900,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="59" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A59">
         <v>58</v>
       </c>
@@ -1917,7 +1914,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="60" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A60">
         <v>59</v>
       </c>
@@ -1931,7 +1928,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="61" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A61">
         <v>60</v>
       </c>
@@ -1945,7 +1942,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="62" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A62">
         <v>61</v>
       </c>
@@ -1959,7 +1956,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="63" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A63">
         <v>62</v>
       </c>
@@ -1973,7 +1970,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="64" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A64">
         <v>63</v>
       </c>
@@ -1987,7 +1984,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="65" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A65">
         <v>64</v>
       </c>
@@ -2001,7 +1998,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="66" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A66">
         <v>65</v>
       </c>
@@ -2015,7 +2012,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="67" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A67">
         <v>66</v>
       </c>
@@ -2029,7 +2026,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="68" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A68">
         <v>67</v>
       </c>
@@ -2043,7 +2040,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="69" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A69">
         <v>68</v>
       </c>
@@ -2057,7 +2054,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="70" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A70">
         <v>69</v>
       </c>
@@ -2071,7 +2068,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="71" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A71">
         <v>70</v>
       </c>
@@ -2085,7 +2082,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="72" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A72">
         <v>71</v>
       </c>
@@ -2099,7 +2096,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="73" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A73">
         <v>72</v>
       </c>
@@ -2113,7 +2110,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="74" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A74">
         <v>73</v>
       </c>
@@ -2127,7 +2124,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="75" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A75">
         <v>74</v>
       </c>
@@ -2141,7 +2138,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="76" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A76">
         <v>75</v>
       </c>
@@ -2155,7 +2152,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="77" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A77">
         <v>76</v>
       </c>
@@ -2169,7 +2166,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="78" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A78">
         <v>77</v>
       </c>
@@ -2183,7 +2180,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="79" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A79">
         <v>78</v>
       </c>
@@ -2197,7 +2194,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="80" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A80">
         <v>79</v>
       </c>
@@ -2211,7 +2208,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="81" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A81">
         <v>80</v>
       </c>
@@ -2225,7 +2222,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="82" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A82">
         <v>81</v>
       </c>
@@ -2239,7 +2236,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="83" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A83">
         <v>82</v>
       </c>
@@ -2253,7 +2250,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="84" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A84">
         <v>83</v>
       </c>
@@ -2267,7 +2264,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="85" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A85">
         <v>84</v>
       </c>
@@ -2281,7 +2278,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="86" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A86">
         <v>85</v>
       </c>
@@ -2295,7 +2292,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="87" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A87">
         <v>86</v>
       </c>
@@ -2309,7 +2306,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="88" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A88">
         <v>87</v>
       </c>
@@ -2323,7 +2320,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="89" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A89">
         <v>88</v>
       </c>
@@ -2337,7 +2334,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="90" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A90">
         <v>89</v>
       </c>
@@ -2351,7 +2348,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="91" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A91">
         <v>90</v>
       </c>
@@ -2365,7 +2362,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="92" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A92">
         <v>91</v>
       </c>
@@ -2379,7 +2376,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="93" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A93">
         <v>92</v>
       </c>
@@ -2393,7 +2390,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="94" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A94">
         <v>93</v>
       </c>
@@ -2407,7 +2404,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="95" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A95">
         <v>94</v>
       </c>
@@ -2421,7 +2418,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="96" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A96">
         <v>95</v>
       </c>
@@ -2444,13 +2441,13 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B7CFBFAA-22DC-428C-A718-7E0BADD40216}">
   <dimension ref="A1:F20"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.44140625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="18.109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="50.88671875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="18.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="50.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>183</v>
       </c>
@@ -2465,7 +2462,7 @@
       </c>
       <c r="E1" s="1"/>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>6</v>
       </c>
@@ -2476,7 +2473,7 @@
         <v>185</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>6</v>
       </c>
@@ -2487,7 +2484,7 @@
         <v>186</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="5" t="s">
         <v>10</v>
       </c>
@@ -2498,7 +2495,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
         <v>10</v>
       </c>
@@ -2509,7 +2506,7 @@
         <v>188</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="5" t="s">
         <v>10</v>
       </c>
@@ -2520,7 +2517,7 @@
         <v>189</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="5" t="s">
         <v>10</v>
       </c>
@@ -2531,7 +2528,7 @@
         <v>190</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="5" t="s">
         <v>10</v>
       </c>
@@ -2542,7 +2539,7 @@
         <v>191</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="5" t="s">
         <v>10</v>
       </c>
@@ -2550,10 +2547,10 @@
         <v>6</v>
       </c>
       <c r="C9" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>12</v>
       </c>
@@ -2564,7 +2561,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>12</v>
       </c>
@@ -2575,7 +2572,7 @@
         <v>188</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>12</v>
       </c>
@@ -2586,7 +2583,7 @@
         <v>189</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>12</v>
       </c>
@@ -2594,10 +2591,10 @@
         <v>4</v>
       </c>
       <c r="C13" s="9" t="s">
-        <v>193</v>
-      </c>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>12</v>
       </c>
@@ -2608,7 +2605,7 @@
         <v>191</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>12</v>
       </c>
@@ -2616,10 +2613,10 @@
         <v>6</v>
       </c>
       <c r="C15" t="s">
-        <v>194</v>
-      </c>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>14</v>
       </c>
@@ -2627,11 +2624,11 @@
         <v>1</v>
       </c>
       <c r="C16" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="F16" s="11"/>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>14</v>
       </c>
@@ -2639,10 +2636,10 @@
         <v>2</v>
       </c>
       <c r="C17" s="9" t="s">
-        <v>196</v>
-      </c>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>14</v>
       </c>
@@ -2650,10 +2647,10 @@
         <v>3</v>
       </c>
       <c r="C18" s="9" t="s">
-        <v>197</v>
-      </c>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>14</v>
       </c>
@@ -2661,10 +2658,10 @@
         <v>4</v>
       </c>
       <c r="C19" s="9" t="s">
-        <v>198</v>
-      </c>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>14</v>
       </c>
@@ -2672,7 +2669,7 @@
         <v>5</v>
       </c>
       <c r="C20" s="9" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
     </row>
   </sheetData>
@@ -2682,6 +2679,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <Zeit xmlns="b63cdcf7-47fa-43f6-87e5-23b415b5c413" xsi:nil="true"/>
@@ -2691,15 +2697,6 @@
     <TaxCatchAll xmlns="12535b08-222e-45d2-b6db-15019f1afee6" xsi:nil="true"/>
   </documentManagement>
 </p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2944,6 +2941,14 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4C05FF1B-7508-40EF-8319-E993EA07F007}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1D9CBEFE-8C4C-4054-8E02-CA457E93B4C8}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
@@ -2956,14 +2961,6 @@
     <ds:schemaRef ds:uri="12535b08-222e-45d2-b6db-15019f1afee6"/>
     <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
     <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4C05FF1B-7508-40EF-8319-E993EA07F007}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>

<commit_message>
GL-5 change in DD Education Variable
</commit_message>
<xml_diff>
--- a/rmonize/data_dictionary/DD_GINI_P1.xlsx
+++ b/rmonize/data_dictionary/DD_GINI_P1.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20417"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="K:\use-cases-harmonisation\rmonize\data_dictionary\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\schwarz-f\Desktop\use-cases-harmonisation\rmonize\data_dictionary\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A0E3838A-CD85-47E3-AEB3-41F2C7F662EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{26FF99F4-00C5-4937-A20C-D9E2912378C7}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="22290" windowHeight="12000" activeTab="1" xr2:uid="{1200B70D-B446-4CDA-99A8-3FD394D791D2}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="331" uniqueCount="212">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="369" uniqueCount="224">
   <si>
     <t>index</t>
   </si>
@@ -663,6 +663,42 @@
   </si>
   <si>
     <t>Number of hours in a normal week (7 days) with heavy physical activity (a lot of sweating, rapid breathing, e.g. ball games, training) in winter [hours]</t>
+  </si>
+  <si>
+    <t>MUTBERU_3</t>
+  </si>
+  <si>
+    <t>VATBERU_3</t>
+  </si>
+  <si>
+    <t>Auszubildende/r, Student/in</t>
+  </si>
+  <si>
+    <t>kein beruflicher Abschluss</t>
+  </si>
+  <si>
+    <t>abgeschlossene beruflich-betriebliche Ausbildung</t>
+  </si>
+  <si>
+    <t>abgeschlossene beruflich-schulische Ausbildung</t>
+  </si>
+  <si>
+    <t>abgeschlossene Ausbildung an Fachschule</t>
+  </si>
+  <si>
+    <t>Fachhochschulabschluss</t>
+  </si>
+  <si>
+    <t>Hochschulabschluss</t>
+  </si>
+  <si>
+    <t>anderer beruflicher Abschluss</t>
+  </si>
+  <si>
+    <t>highest job qualification of the mother</t>
+  </si>
+  <si>
+    <t>highest job qualification of the father</t>
   </si>
 </sst>
 </file>
@@ -731,7 +767,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -766,9 +802,12 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Standard" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -784,9 +823,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office">
   <a:themeElements>
-    <a:clrScheme name="Office 2013 - 2022">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -824,7 +863,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2013 - 2022">
+    <a:fontScheme name="Office">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -930,7 +969,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2013 - 2022">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1072,7 +1111,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -1080,8 +1119,8 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{08A73012-5CAD-43B9-A281-79101DF4E1E0}">
-  <dimension ref="A1:D96"/>
-  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:D98"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="19.140625" customWidth="1"/>
     <col min="3" max="3" width="53.42578125" bestFit="1" customWidth="1"/>
@@ -1177,13 +1216,13 @@
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>200</v>
+        <v>212</v>
       </c>
       <c r="C7" t="s">
-        <v>201</v>
-      </c>
-      <c r="D7" t="s">
-        <v>18</v>
+        <v>222</v>
+      </c>
+      <c r="D7" s="11" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
@@ -1191,13 +1230,13 @@
         <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>202</v>
-      </c>
-      <c r="C8" t="s">
-        <v>203</v>
-      </c>
-      <c r="D8" t="s">
-        <v>18</v>
+        <v>213</v>
+      </c>
+      <c r="C8" s="8" t="s">
+        <v>223</v>
+      </c>
+      <c r="D8" s="11" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
@@ -1205,10 +1244,10 @@
         <v>8</v>
       </c>
       <c r="B9" t="s">
-        <v>204</v>
+        <v>200</v>
       </c>
       <c r="C9" t="s">
-        <v>205</v>
+        <v>201</v>
       </c>
       <c r="D9" t="s">
         <v>18</v>
@@ -1219,10 +1258,10 @@
         <v>9</v>
       </c>
       <c r="B10" t="s">
-        <v>206</v>
+        <v>202</v>
       </c>
       <c r="C10" t="s">
-        <v>207</v>
+        <v>203</v>
       </c>
       <c r="D10" t="s">
         <v>18</v>
@@ -1233,10 +1272,10 @@
         <v>10</v>
       </c>
       <c r="B11" t="s">
-        <v>208</v>
+        <v>204</v>
       </c>
       <c r="C11" t="s">
-        <v>209</v>
+        <v>205</v>
       </c>
       <c r="D11" t="s">
         <v>18</v>
@@ -1247,10 +1286,10 @@
         <v>11</v>
       </c>
       <c r="B12" t="s">
-        <v>210</v>
+        <v>206</v>
       </c>
       <c r="C12" t="s">
-        <v>211</v>
+        <v>207</v>
       </c>
       <c r="D12" t="s">
         <v>18</v>
@@ -1260,27 +1299,27 @@
       <c r="A13">
         <v>12</v>
       </c>
-      <c r="B13" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="C13" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="D13" s="3" t="s">
-        <v>5</v>
+      <c r="B13" t="s">
+        <v>208</v>
+      </c>
+      <c r="C13" t="s">
+        <v>209</v>
+      </c>
+      <c r="D13" t="s">
+        <v>18</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>13</v>
       </c>
-      <c r="B14" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="C14" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="D14" s="6" t="s">
+      <c r="B14" t="s">
+        <v>210</v>
+      </c>
+      <c r="C14" t="s">
+        <v>211</v>
+      </c>
+      <c r="D14" t="s">
         <v>18</v>
       </c>
     </row>
@@ -1288,27 +1327,27 @@
       <c r="A15">
         <v>14</v>
       </c>
-      <c r="B15" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="C15" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="D15" s="6" t="s">
-        <v>18</v>
+      <c r="B15" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C15" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="D15" s="3" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>15</v>
       </c>
-      <c r="B16" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="C16" t="s">
-        <v>22</v>
-      </c>
-      <c r="D16" t="s">
+      <c r="B16" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="C16" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="D16" s="6" t="s">
         <v>18</v>
       </c>
     </row>
@@ -1316,13 +1355,13 @@
       <c r="A17">
         <v>16</v>
       </c>
-      <c r="B17" s="7" t="s">
-        <v>23</v>
-      </c>
-      <c r="C17" t="s">
-        <v>24</v>
-      </c>
-      <c r="D17" t="s">
+      <c r="B17" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="C17" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="D17" s="6" t="s">
         <v>18</v>
       </c>
     </row>
@@ -1330,11 +1369,11 @@
       <c r="A18">
         <v>17</v>
       </c>
-      <c r="B18" s="3" t="s">
-        <v>25</v>
+      <c r="B18" s="7" t="s">
+        <v>21</v>
       </c>
       <c r="C18" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="D18" t="s">
         <v>18</v>
@@ -1344,11 +1383,11 @@
       <c r="A19">
         <v>18</v>
       </c>
-      <c r="B19" s="3" t="s">
-        <v>27</v>
+      <c r="B19" s="7" t="s">
+        <v>23</v>
       </c>
       <c r="C19" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="D19" t="s">
         <v>18</v>
@@ -1359,10 +1398,10 @@
         <v>19</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="C20" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="D20" t="s">
         <v>18</v>
@@ -1373,10 +1412,10 @@
         <v>20</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="C21" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="D21" t="s">
         <v>18</v>
@@ -1387,10 +1426,10 @@
         <v>21</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="C22" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="D22" t="s">
         <v>18</v>
@@ -1401,10 +1440,10 @@
         <v>22</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="C23" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="D23" t="s">
         <v>18</v>
@@ -1415,10 +1454,10 @@
         <v>23</v>
       </c>
       <c r="B24" s="3" t="s">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="C24" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="D24" t="s">
         <v>18</v>
@@ -1429,10 +1468,10 @@
         <v>24</v>
       </c>
       <c r="B25" s="3" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="C25" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="D25" t="s">
         <v>18</v>
@@ -1443,10 +1482,10 @@
         <v>25</v>
       </c>
       <c r="B26" s="3" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="C26" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="D26" t="s">
         <v>18</v>
@@ -1457,10 +1496,10 @@
         <v>26</v>
       </c>
       <c r="B27" s="3" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="C27" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="D27" t="s">
         <v>18</v>
@@ -1471,10 +1510,10 @@
         <v>27</v>
       </c>
       <c r="B28" s="3" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="C28" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="D28" t="s">
         <v>18</v>
@@ -1485,10 +1524,10 @@
         <v>28</v>
       </c>
       <c r="B29" s="3" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="C29" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="D29" t="s">
         <v>18</v>
@@ -1499,10 +1538,10 @@
         <v>29</v>
       </c>
       <c r="B30" s="3" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="C30" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="D30" t="s">
         <v>18</v>
@@ -1513,10 +1552,10 @@
         <v>30</v>
       </c>
       <c r="B31" s="3" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="C31" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="D31" t="s">
         <v>18</v>
@@ -1527,10 +1566,10 @@
         <v>31</v>
       </c>
       <c r="B32" s="3" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="C32" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="D32" t="s">
         <v>18</v>
@@ -1541,10 +1580,10 @@
         <v>32</v>
       </c>
       <c r="B33" s="3" t="s">
-        <v>55</v>
-      </c>
-      <c r="C33" s="3" t="s">
-        <v>56</v>
+        <v>51</v>
+      </c>
+      <c r="C33" t="s">
+        <v>52</v>
       </c>
       <c r="D33" t="s">
         <v>18</v>
@@ -1555,10 +1594,10 @@
         <v>33</v>
       </c>
       <c r="B34" s="3" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="C34" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="D34" t="s">
         <v>18</v>
@@ -1569,10 +1608,10 @@
         <v>34</v>
       </c>
       <c r="B35" s="3" t="s">
-        <v>59</v>
-      </c>
-      <c r="C35" t="s">
-        <v>60</v>
+        <v>55</v>
+      </c>
+      <c r="C35" s="3" t="s">
+        <v>56</v>
       </c>
       <c r="D35" t="s">
         <v>18</v>
@@ -1583,10 +1622,10 @@
         <v>35</v>
       </c>
       <c r="B36" s="3" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="C36" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="D36" t="s">
         <v>18</v>
@@ -1596,11 +1635,11 @@
       <c r="A37">
         <v>36</v>
       </c>
-      <c r="B37" t="s">
-        <v>63</v>
+      <c r="B37" s="3" t="s">
+        <v>59</v>
       </c>
       <c r="C37" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="D37" t="s">
         <v>18</v>
@@ -1610,11 +1649,11 @@
       <c r="A38">
         <v>37</v>
       </c>
-      <c r="B38" t="s">
-        <v>65</v>
+      <c r="B38" s="3" t="s">
+        <v>61</v>
       </c>
       <c r="C38" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="D38" t="s">
         <v>18</v>
@@ -1625,10 +1664,10 @@
         <v>38</v>
       </c>
       <c r="B39" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="C39" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="D39" t="s">
         <v>18</v>
@@ -1639,10 +1678,10 @@
         <v>39</v>
       </c>
       <c r="B40" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
       <c r="C40" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="D40" t="s">
         <v>18</v>
@@ -1653,10 +1692,10 @@
         <v>40</v>
       </c>
       <c r="B41" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="C41" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="D41" t="s">
         <v>18</v>
@@ -1667,10 +1706,10 @@
         <v>41</v>
       </c>
       <c r="B42" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="C42" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="D42" t="s">
         <v>18</v>
@@ -1681,10 +1720,10 @@
         <v>42</v>
       </c>
       <c r="B43" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="C43" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="D43" t="s">
         <v>18</v>
@@ -1695,10 +1734,10 @@
         <v>43</v>
       </c>
       <c r="B44" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="C44" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="D44" t="s">
         <v>18</v>
@@ -1709,10 +1748,10 @@
         <v>44</v>
       </c>
       <c r="B45" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="C45" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="D45" t="s">
         <v>18</v>
@@ -1723,10 +1762,10 @@
         <v>45</v>
       </c>
       <c r="B46" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="C46" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="D46" t="s">
         <v>18</v>
@@ -1737,10 +1776,10 @@
         <v>46</v>
       </c>
       <c r="B47" t="s">
-        <v>83</v>
-      </c>
-      <c r="C47" s="13" t="s">
-        <v>84</v>
+        <v>79</v>
+      </c>
+      <c r="C47" t="s">
+        <v>80</v>
       </c>
       <c r="D47" t="s">
         <v>18</v>
@@ -1751,10 +1790,10 @@
         <v>47</v>
       </c>
       <c r="B48" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="C48" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
       <c r="D48" t="s">
         <v>18</v>
@@ -1765,10 +1804,10 @@
         <v>48</v>
       </c>
       <c r="B49" t="s">
-        <v>87</v>
-      </c>
-      <c r="C49" t="s">
-        <v>88</v>
+        <v>83</v>
+      </c>
+      <c r="C49" s="13" t="s">
+        <v>84</v>
       </c>
       <c r="D49" t="s">
         <v>18</v>
@@ -1779,10 +1818,10 @@
         <v>49</v>
       </c>
       <c r="B50" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="C50" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="D50" t="s">
         <v>18</v>
@@ -1793,10 +1832,10 @@
         <v>50</v>
       </c>
       <c r="B51" t="s">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="C51" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="D51" t="s">
         <v>18</v>
@@ -1807,10 +1846,10 @@
         <v>51</v>
       </c>
       <c r="B52" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="C52" t="s">
-        <v>94</v>
+        <v>90</v>
       </c>
       <c r="D52" t="s">
         <v>18</v>
@@ -1821,10 +1860,10 @@
         <v>52</v>
       </c>
       <c r="B53" t="s">
-        <v>95</v>
+        <v>91</v>
       </c>
       <c r="C53" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="D53" t="s">
         <v>18</v>
@@ -1835,10 +1874,10 @@
         <v>53</v>
       </c>
       <c r="B54" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="C54" t="s">
-        <v>98</v>
+        <v>94</v>
       </c>
       <c r="D54" t="s">
         <v>18</v>
@@ -1848,11 +1887,11 @@
       <c r="A55">
         <v>54</v>
       </c>
-      <c r="B55" s="3" t="s">
-        <v>99</v>
+      <c r="B55" t="s">
+        <v>95</v>
       </c>
       <c r="C55" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="D55" t="s">
         <v>18</v>
@@ -1863,10 +1902,10 @@
         <v>55</v>
       </c>
       <c r="B56" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="C56" t="s">
-        <v>102</v>
+        <v>98</v>
       </c>
       <c r="D56" t="s">
         <v>18</v>
@@ -1876,11 +1915,11 @@
       <c r="A57">
         <v>56</v>
       </c>
-      <c r="B57" t="s">
-        <v>103</v>
+      <c r="B57" s="3" t="s">
+        <v>99</v>
       </c>
       <c r="C57" t="s">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="D57" t="s">
         <v>18</v>
@@ -1891,10 +1930,10 @@
         <v>57</v>
       </c>
       <c r="B58" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
       <c r="C58" t="s">
-        <v>106</v>
+        <v>102</v>
       </c>
       <c r="D58" t="s">
         <v>18</v>
@@ -1905,10 +1944,10 @@
         <v>58</v>
       </c>
       <c r="B59" t="s">
-        <v>107</v>
+        <v>103</v>
       </c>
       <c r="C59" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="D59" t="s">
         <v>18</v>
@@ -1919,10 +1958,10 @@
         <v>59</v>
       </c>
       <c r="B60" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="C60" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="D60" t="s">
         <v>18</v>
@@ -1933,10 +1972,10 @@
         <v>60</v>
       </c>
       <c r="B61" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="C61" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="D61" t="s">
         <v>18</v>
@@ -1947,10 +1986,10 @@
         <v>61</v>
       </c>
       <c r="B62" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="C62" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="D62" t="s">
         <v>18</v>
@@ -1961,10 +2000,10 @@
         <v>62</v>
       </c>
       <c r="B63" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="C63" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
       <c r="D63" t="s">
         <v>18</v>
@@ -1975,10 +2014,10 @@
         <v>63</v>
       </c>
       <c r="B64" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="C64" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="D64" t="s">
         <v>18</v>
@@ -1989,10 +2028,10 @@
         <v>64</v>
       </c>
       <c r="B65" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="C65" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="D65" t="s">
         <v>18</v>
@@ -2003,10 +2042,10 @@
         <v>65</v>
       </c>
       <c r="B66" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="C66" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="D66" t="s">
         <v>18</v>
@@ -2017,10 +2056,10 @@
         <v>66</v>
       </c>
       <c r="B67" t="s">
-        <v>123</v>
+        <v>119</v>
       </c>
       <c r="C67" t="s">
-        <v>124</v>
+        <v>120</v>
       </c>
       <c r="D67" t="s">
         <v>18</v>
@@ -2031,10 +2070,10 @@
         <v>67</v>
       </c>
       <c r="B68" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="C68" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="D68" t="s">
         <v>18</v>
@@ -2045,10 +2084,10 @@
         <v>68</v>
       </c>
       <c r="B69" t="s">
-        <v>127</v>
+        <v>123</v>
       </c>
       <c r="C69" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
       <c r="D69" t="s">
         <v>18</v>
@@ -2059,10 +2098,10 @@
         <v>69</v>
       </c>
       <c r="B70" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
       <c r="C70" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="D70" t="s">
         <v>18</v>
@@ -2073,10 +2112,10 @@
         <v>70</v>
       </c>
       <c r="B71" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
       <c r="C71" t="s">
-        <v>132</v>
+        <v>128</v>
       </c>
       <c r="D71" t="s">
         <v>18</v>
@@ -2087,10 +2126,10 @@
         <v>71</v>
       </c>
       <c r="B72" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="C72" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
       <c r="D72" t="s">
         <v>18</v>
@@ -2101,10 +2140,10 @@
         <v>72</v>
       </c>
       <c r="B73" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="C73" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="D73" t="s">
         <v>18</v>
@@ -2115,10 +2154,10 @@
         <v>73</v>
       </c>
       <c r="B74" t="s">
-        <v>137</v>
+        <v>133</v>
       </c>
       <c r="C74" t="s">
-        <v>138</v>
+        <v>134</v>
       </c>
       <c r="D74" t="s">
         <v>18</v>
@@ -2129,10 +2168,10 @@
         <v>74</v>
       </c>
       <c r="B75" t="s">
-        <v>139</v>
+        <v>135</v>
       </c>
       <c r="C75" t="s">
-        <v>140</v>
+        <v>136</v>
       </c>
       <c r="D75" t="s">
         <v>18</v>
@@ -2143,10 +2182,10 @@
         <v>75</v>
       </c>
       <c r="B76" t="s">
-        <v>141</v>
+        <v>137</v>
       </c>
       <c r="C76" t="s">
-        <v>142</v>
+        <v>138</v>
       </c>
       <c r="D76" t="s">
         <v>18</v>
@@ -2157,10 +2196,10 @@
         <v>76</v>
       </c>
       <c r="B77" t="s">
-        <v>143</v>
+        <v>139</v>
       </c>
       <c r="C77" t="s">
-        <v>144</v>
+        <v>140</v>
       </c>
       <c r="D77" t="s">
         <v>18</v>
@@ -2171,10 +2210,10 @@
         <v>77</v>
       </c>
       <c r="B78" t="s">
-        <v>145</v>
+        <v>141</v>
       </c>
       <c r="C78" t="s">
-        <v>146</v>
+        <v>142</v>
       </c>
       <c r="D78" t="s">
         <v>18</v>
@@ -2185,10 +2224,10 @@
         <v>78</v>
       </c>
       <c r="B79" t="s">
-        <v>147</v>
+        <v>143</v>
       </c>
       <c r="C79" t="s">
-        <v>148</v>
+        <v>144</v>
       </c>
       <c r="D79" t="s">
         <v>18</v>
@@ -2199,10 +2238,10 @@
         <v>79</v>
       </c>
       <c r="B80" t="s">
-        <v>149</v>
+        <v>145</v>
       </c>
       <c r="C80" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
       <c r="D80" t="s">
         <v>18</v>
@@ -2213,10 +2252,10 @@
         <v>80</v>
       </c>
       <c r="B81" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="C81" t="s">
-        <v>152</v>
+        <v>148</v>
       </c>
       <c r="D81" t="s">
         <v>18</v>
@@ -2227,10 +2266,10 @@
         <v>81</v>
       </c>
       <c r="B82" t="s">
-        <v>153</v>
+        <v>149</v>
       </c>
       <c r="C82" t="s">
-        <v>154</v>
+        <v>150</v>
       </c>
       <c r="D82" t="s">
         <v>18</v>
@@ -2241,10 +2280,10 @@
         <v>82</v>
       </c>
       <c r="B83" t="s">
-        <v>155</v>
+        <v>151</v>
       </c>
       <c r="C83" t="s">
-        <v>156</v>
+        <v>152</v>
       </c>
       <c r="D83" t="s">
         <v>18</v>
@@ -2255,10 +2294,10 @@
         <v>83</v>
       </c>
       <c r="B84" t="s">
-        <v>157</v>
+        <v>153</v>
       </c>
       <c r="C84" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
       <c r="D84" t="s">
         <v>18</v>
@@ -2269,10 +2308,10 @@
         <v>84</v>
       </c>
       <c r="B85" t="s">
-        <v>159</v>
+        <v>155</v>
       </c>
       <c r="C85" t="s">
-        <v>160</v>
+        <v>156</v>
       </c>
       <c r="D85" t="s">
         <v>18</v>
@@ -2283,10 +2322,10 @@
         <v>85</v>
       </c>
       <c r="B86" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
       <c r="C86" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
       <c r="D86" t="s">
         <v>18</v>
@@ -2297,10 +2336,10 @@
         <v>86</v>
       </c>
       <c r="B87" t="s">
-        <v>163</v>
+        <v>159</v>
       </c>
       <c r="C87" t="s">
-        <v>164</v>
+        <v>160</v>
       </c>
       <c r="D87" t="s">
         <v>18</v>
@@ -2311,10 +2350,10 @@
         <v>87</v>
       </c>
       <c r="B88" t="s">
-        <v>165</v>
+        <v>161</v>
       </c>
       <c r="C88" t="s">
-        <v>166</v>
+        <v>162</v>
       </c>
       <c r="D88" t="s">
         <v>18</v>
@@ -2325,10 +2364,10 @@
         <v>88</v>
       </c>
       <c r="B89" t="s">
-        <v>167</v>
+        <v>163</v>
       </c>
       <c r="C89" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="D89" t="s">
         <v>18</v>
@@ -2339,10 +2378,10 @@
         <v>89</v>
       </c>
       <c r="B90" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
       <c r="C90" t="s">
-        <v>170</v>
+        <v>166</v>
       </c>
       <c r="D90" t="s">
         <v>18</v>
@@ -2352,11 +2391,11 @@
       <c r="A91">
         <v>90</v>
       </c>
-      <c r="B91" s="3" t="s">
-        <v>171</v>
+      <c r="B91" t="s">
+        <v>167</v>
       </c>
       <c r="C91" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="D91" t="s">
         <v>18</v>
@@ -2366,11 +2405,11 @@
       <c r="A92">
         <v>91</v>
       </c>
-      <c r="B92" s="3" t="s">
-        <v>173</v>
+      <c r="B92" t="s">
+        <v>169</v>
       </c>
       <c r="C92" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
       <c r="D92" t="s">
         <v>18</v>
@@ -2381,10 +2420,10 @@
         <v>92</v>
       </c>
       <c r="B93" s="3" t="s">
-        <v>175</v>
+        <v>171</v>
       </c>
       <c r="C93" t="s">
-        <v>176</v>
+        <v>172</v>
       </c>
       <c r="D93" t="s">
         <v>18</v>
@@ -2394,11 +2433,11 @@
       <c r="A94">
         <v>93</v>
       </c>
-      <c r="B94" t="s">
-        <v>177</v>
+      <c r="B94" s="3" t="s">
+        <v>173</v>
       </c>
       <c r="C94" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="D94" t="s">
         <v>18</v>
@@ -2408,11 +2447,11 @@
       <c r="A95">
         <v>94</v>
       </c>
-      <c r="B95" t="s">
-        <v>179</v>
-      </c>
-      <c r="C95" s="12" t="s">
-        <v>180</v>
+      <c r="B95" s="3" t="s">
+        <v>175</v>
+      </c>
+      <c r="C95" t="s">
+        <v>176</v>
       </c>
       <c r="D95" t="s">
         <v>18</v>
@@ -2422,13 +2461,41 @@
       <c r="A96">
         <v>95</v>
       </c>
-      <c r="B96" s="3" t="s">
+      <c r="B96" t="s">
+        <v>177</v>
+      </c>
+      <c r="C96" t="s">
+        <v>178</v>
+      </c>
+      <c r="D96" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="97" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A97">
+        <v>96</v>
+      </c>
+      <c r="B97" t="s">
+        <v>179</v>
+      </c>
+      <c r="C97" s="12" t="s">
+        <v>180</v>
+      </c>
+      <c r="D97" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="98" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A98">
+        <v>97</v>
+      </c>
+      <c r="B98" s="3" t="s">
         <v>181</v>
       </c>
-      <c r="C96" t="s">
+      <c r="C98" t="s">
         <v>182</v>
       </c>
-      <c r="D96" t="s">
+      <c r="D98" t="s">
         <v>18</v>
       </c>
     </row>
@@ -2440,8 +2507,8 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B7CFBFAA-22DC-428C-A718-7E0BADD40216}">
-  <dimension ref="A1:F20"/>
-  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:F36"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="18.140625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="50.85546875" bestFit="1" customWidth="1"/>
@@ -2672,6 +2739,182 @@
         <v>198</v>
       </c>
     </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>212</v>
+      </c>
+      <c r="B21" s="10">
+        <v>1</v>
+      </c>
+      <c r="C21" s="14" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>212</v>
+      </c>
+      <c r="B22" s="10">
+        <v>2</v>
+      </c>
+      <c r="C22" s="14" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>212</v>
+      </c>
+      <c r="B23" s="10">
+        <v>3</v>
+      </c>
+      <c r="C23" s="14" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>212</v>
+      </c>
+      <c r="B24" s="10">
+        <v>4</v>
+      </c>
+      <c r="C24" s="14" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>212</v>
+      </c>
+      <c r="B25" s="10">
+        <v>5</v>
+      </c>
+      <c r="C25" s="14" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>212</v>
+      </c>
+      <c r="B26" s="10">
+        <v>6</v>
+      </c>
+      <c r="C26" s="14" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>212</v>
+      </c>
+      <c r="B27" s="10">
+        <v>7</v>
+      </c>
+      <c r="C27" s="14" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>212</v>
+      </c>
+      <c r="B28" s="10">
+        <v>8</v>
+      </c>
+      <c r="C28" s="14" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>213</v>
+      </c>
+      <c r="B29" s="10">
+        <v>1</v>
+      </c>
+      <c r="C29" s="14" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>213</v>
+      </c>
+      <c r="B30" s="10">
+        <v>2</v>
+      </c>
+      <c r="C30" s="14" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>213</v>
+      </c>
+      <c r="B31" s="10">
+        <v>3</v>
+      </c>
+      <c r="C31" s="14" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>213</v>
+      </c>
+      <c r="B32" s="10">
+        <v>4</v>
+      </c>
+      <c r="C32" s="14" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>213</v>
+      </c>
+      <c r="B33" s="10">
+        <v>5</v>
+      </c>
+      <c r="C33" s="14" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>213</v>
+      </c>
+      <c r="B34" s="10">
+        <v>6</v>
+      </c>
+      <c r="C34" s="14" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>213</v>
+      </c>
+      <c r="B35" s="10">
+        <v>7</v>
+      </c>
+      <c r="C35" s="14" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>213</v>
+      </c>
+      <c r="B36" s="10">
+        <v>8</v>
+      </c>
+      <c r="C36" s="14" t="s">
+        <v>221</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -2679,15 +2922,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <Zeit xmlns="b63cdcf7-47fa-43f6-87e5-23b415b5c413" xsi:nil="true"/>
@@ -2697,6 +2931,15 @@
     <TaxCatchAll xmlns="12535b08-222e-45d2-b6db-15019f1afee6" xsi:nil="true"/>
   </documentManagement>
 </p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2941,14 +3184,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4C05FF1B-7508-40EF-8319-E993EA07F007}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1D9CBEFE-8C4C-4054-8E02-CA457E93B4C8}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
@@ -2961,6 +3196,14 @@
     <ds:schemaRef ds:uri="12535b08-222e-45d2-b6db-15019f1afee6"/>
     <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
     <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4C05FF1B-7508-40EF-8319-E993EA07F007}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>